<commit_message>
Added first annnouncement for BBS Annual Meeting 2026: Quantitative drug development in the age of AI (on Nov 10th, 2026)
</commit_message>
<xml_diff>
--- a/data/upcoming.xlsx
+++ b/data/upcoming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schaej17\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CC27D8-D69E-4A06-9281-7EF22823B6A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE31CAB-33EC-4C9C-A445-B987909D6D35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>date</t>
   </si>
@@ -78,6 +78,12 @@
   </si>
   <si>
     <t>https://forms.cloud.microsoft/r/VA3QdVjrZ5</t>
+  </si>
+  <si>
+    <t>Quantitative drug development in the age of AI</t>
+  </si>
+  <si>
+    <t>Annual Meeting</t>
   </si>
 </sst>
 </file>
@@ -497,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E916"/>
+  <dimension ref="A1:E917"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" style="9" bestFit="1" customWidth="1"/>
@@ -540,35 +546,43 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="str">
+        <f>"10.11.2026"</f>
+        <v>10.11.2026</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="str">
         <f>"01.12.2026"</f>
         <v>01.12.2026</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D4" s="12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B6" s="4"/>
@@ -578,12 +592,12 @@
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="5"/>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B8" s="4"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B9" s="4"/>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="5"/>
       <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -591,8 +605,8 @@
       <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B12" s="3"/>
@@ -606,13 +620,13 @@
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="3"/>
@@ -643,8 +657,8 @@
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B25" s="4"/>
@@ -1099,9 +1113,8 @@
       <c r="C137" s="4"/>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A138" s="10"/>
-      <c r="B138" s="7"/>
-      <c r="C138" s="7"/>
+      <c r="B138" s="4"/>
+      <c r="C138" s="4"/>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" s="10"/>
@@ -4993,9 +5006,14 @@
       <c r="B916" s="7"/>
       <c r="C916" s="7"/>
     </row>
+    <row r="917" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A917" s="10"/>
+      <c r="B917" s="7"/>
+      <c r="C917" s="7"/>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" xr:uid="{A101E298-53BC-4B3C-A6DD-AE4DCA3328DF}"/>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{A101E298-53BC-4B3C-A6DD-AE4DCA3328DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>